<commit_message>
v2.1: Update OSP Budget Template to 1/30/2026; NIH salary cap to $228,000; remove PII
</commit_message>
<xml_diff>
--- a/su-osp-budget/assets/OSP-Budget-Template-FY-26-Web.xlsx
+++ b/su-osp-budget/assets/OSP-Budget-Template-FY-26-Web.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\AAF\OSP\OSP Responsibilities - External\Proposal Submission\4.0_Budget_Development\Budget Tools\For Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{342A01B1-B30F-4A1E-8204-78D640FE3CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F80A92AA-0789-4F00-8413-9DA26A5CD594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="IgFBuO7fCmw9GMKIrE1/wNxJXmBD9G+mQLxtrisdZ1VGF28qTncKvGp0iJdbS4WHt/3t8O0AOfJVSgaXVvBeMQ==" workbookSaltValue="/UbcMGXxfNe9+q2MCd7kPA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="5040" windowWidth="18900" windowHeight="11055" tabRatio="929" firstSheet="1" activeTab="3" xr2:uid="{10EBF69F-CDF4-4325-BD3F-B84054EE4520}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="929" firstSheet="1" activeTab="1" xr2:uid="{10EBF69F-CDF4-4325-BD3F-B84054EE4520}"/>
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="20" state="hidden" r:id="rId1"/>
@@ -129,7 +130,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2239" uniqueCount="679">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2240" uniqueCount="680">
   <si>
     <t>Prefix</t>
   </si>
@@ -2378,9 +2379,6 @@
     <t>File Copy and File Copy-No Salary tabs - fixed problem with year five and Other personnel fringe.</t>
   </si>
   <si>
-    <t>FY24 - $1,872</t>
-  </si>
-  <si>
     <t>3/21/20224</t>
   </si>
   <si>
@@ -2399,7 +2397,13 @@
     <t>Directions for Completing the OSP Campus R&amp;R Budget Template - FY 26</t>
   </si>
   <si>
-    <t>Last Updated: 7/2/2025</t>
+    <t>FY26 - $2,015</t>
+  </si>
+  <si>
+    <t>Update to NIH Salary Cap</t>
+  </si>
+  <si>
+    <t>Last Updated: 1/30/2026</t>
   </si>
 </sst>
 </file>
@@ -7072,7 +7076,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
-  <dimension ref="A1:A159"/>
+  <dimension ref="A1:A162"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -7080,37 +7084,37 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="58">
-        <v>45840</v>
+        <v>46052</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="273" t="s">
-        <v>522</v>
+      <c r="A2" t="s">
+        <v>678</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="58">
-        <v>45831</v>
+        <v>45840</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="58">
-        <v>45456</v>
+        <v>45831</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="58">
-        <v>45394</v>
+        <v>45456</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
@@ -7119,525 +7123,535 @@
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>672</v>
+      <c r="A13" s="58">
+        <v>45394</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" s="58">
-        <v>45324</v>
+      <c r="A16" t="s">
+        <v>671</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="273" t="s">
-        <v>522</v>
+      <c r="A17" t="s">
+        <v>672</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="58">
+        <v>45324</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="273" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="58">
         <v>45218</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" s="58">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="58">
         <v>45146</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="460" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="460" t="s">
         <v>667</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="273" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="273" t="s">
         <v>668</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="273" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="273" t="s">
         <v>669</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" s="58">
-        <v>45138</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>666</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" s="58">
+        <v>45138</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="58">
         <v>45135</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" s="273" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="273" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A34" s="273" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" s="273" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="273" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" s="273" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" s="273" t="s">
         <v>665</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" s="273"/>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37" s="58">
-        <v>45117</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>582</v>
-      </c>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" s="273"/>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" s="58">
-        <v>45112</v>
+        <v>45117</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" s="58">
-        <v>45106</v>
+        <v>45112</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" s="58">
+        <v>45106</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>579</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A47" s="58">
-        <v>45105</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" s="58">
-        <v>45104</v>
+        <v>45105</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A53" s="58" t="s">
-        <v>572</v>
+      <c r="A53" s="58">
+        <v>45104</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A56" s="58" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>543</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>544</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A58" s="58">
-        <v>45027</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A59" s="273" t="s">
-        <v>526</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" s="58">
-        <v>45009</v>
+        <v>45027</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>524</v>
+      <c r="A62" s="273" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" s="58">
+        <v>45009</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" s="58">
         <v>45007</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A65" s="273" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" s="273" t="s">
         <v>521</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A66" s="273" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A68" s="58">
-        <v>44714</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" s="273" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A71" s="58">
+        <v>44714</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A72" s="273" t="s">
         <v>518</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A70" s="273" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A72" s="58">
-        <v>44617</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A73" s="273" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A75" s="58">
-        <v>44364</v>
+        <v>44617</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A76" s="273" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A78" s="58">
-        <v>44236</v>
+        <v>44364</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>514</v>
+      <c r="A79" s="273" t="s">
+        <v>515</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" s="58">
-        <v>44005</v>
+        <v>44236</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A84" s="58">
-        <v>43986</v>
+        <v>44005</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A87" s="58">
+        <v>43986</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A90" s="58">
         <v>43985</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A88" s="273" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A89" s="273" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A90" s="273" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" s="273" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A92" s="273" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A93" s="273" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A94" s="273" t="s">
         <v>511</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A93" s="58">
-        <v>43682</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A96" s="58">
-        <v>43679</v>
+        <v>43682</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A99" s="58">
-        <v>43656</v>
+        <v>43679</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A100" s="58" t="s">
-        <v>505</v>
+      <c r="A100" t="s">
+        <v>506</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A102" s="58">
-        <v>43206</v>
+        <v>43656</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A103" s="273" t="s">
-        <v>503</v>
+      <c r="A103" s="58" t="s">
+        <v>505</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A105" s="58">
-        <v>43150</v>
+        <v>43206</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
-        <v>502</v>
+      <c r="A106" s="273" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A108" s="58">
-        <v>43020</v>
+        <v>43150</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A109" s="273" t="s">
-        <v>501</v>
+      <c r="A109" t="s">
+        <v>502</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A111" s="58">
-        <v>42831</v>
+        <v>43020</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
-        <v>500</v>
+      <c r="A112" s="273" t="s">
+        <v>501</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A114" s="58">
-        <v>42767</v>
+        <v>42831</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A115" s="273" t="s">
-        <v>499</v>
+      <c r="A115" t="s">
+        <v>500</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A117" s="58">
+        <v>42767</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A118" s="273" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A120" s="58">
         <v>42425</v>
       </c>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A118" t="s">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
         <v>497</v>
-      </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A119" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A121" s="58">
-        <v>42375</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A124" s="58">
-        <v>42193</v>
+        <v>42375</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A127" s="58">
-        <v>42192</v>
+        <v>42193</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A130" s="58">
-        <v>42094</v>
+        <v>42192</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A133" s="58">
+        <v>42094</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
         <v>490</v>
-      </c>
-    </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A132" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A134" s="58">
-        <v>42047</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A137" s="58">
-        <v>42037</v>
+        <v>42047</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A140" s="58">
-        <v>42034</v>
+        <v>42037</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A143" s="58">
+        <v>42034</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
         <v>485</v>
       </c>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A142" t="s">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A145" t="s">
         <v>486</v>
-      </c>
-    </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A144" s="58">
-        <v>41681</v>
-      </c>
-    </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A145" s="273" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A147" s="58">
+        <v>41681</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A148" s="273" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A150" s="58">
         <v>41674</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A148" t="s">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A149" t="s">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A152" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A151" s="58">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A154" s="58">
         <v>40645</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A152" s="24" t="s">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A155" s="24" t="s">
         <v>387</v>
-      </c>
-    </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A153" s="24" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A155" s="58">
-        <v>40641</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A156" s="24" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A158" s="58">
-        <v>40632</v>
+        <v>40641</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A159" s="24" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A161" s="58">
+        <v>40632</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A162" s="24" t="s">
         <v>389</v>
       </c>
     </row>
@@ -28030,7 +28044,7 @@
         <v>1872</v>
       </c>
       <c r="P2" s="273" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="Q2" s="273">
         <v>0</v>
@@ -28085,7 +28099,7 @@
       </c>
       <c r="P3" s="273"/>
       <c r="Q3" s="328">
-        <v>225700</v>
+        <v>228000</v>
       </c>
       <c r="S3" s="273" t="s">
         <v>529</v>
@@ -28173,7 +28187,7 @@
         <v>0.35</v>
       </c>
       <c r="M5" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="N5">
         <v>4</v>
@@ -34592,7 +34606,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="478" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B1" s="478"/>
       <c r="C1" s="478"/>
@@ -34616,7 +34630,7 @@
     </row>
     <row r="3" spans="1:8" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A3" s="479" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B3" s="479"/>
       <c r="C3" s="479"/>
@@ -35918,7 +35932,7 @@
       <c r="F93" s="457"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="ibJipJrIaFSm+Zlkr0WiDY02GypzFqs4vEZ4diSN4tdabVQfRUuDC7rvYjW4KPbDwOHMMXRDGSeIdOwInNoW7w==" saltValue="HAPCANsnqiz0p8f2X+LW4g==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="SjJi4UCvbKB2eoaO4AO+xB9xp4q8NyRyasOHTMPbsQ+E9b+2F6rPDoRJZ+doO6F/maL9zEdJrC7Ag+w6fnlKOw==" saltValue="HR61ly4nzzzRSsfGDg8zlw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="51">
     <mergeCell ref="B11:H11"/>
     <mergeCell ref="B26:H26"/>
@@ -40049,7 +40063,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="rtssKXtBu4qoj81reOvsEZLbUCElLgmaFlaZS74KJKsvbTY+RwGtNSy4+TNvmsgDPk7TDuyMKDdYNUv7+cnZFw==" saltValue="o1CdZ1J1hqM9mX/PnGFNyQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="jFdV4oL2D3Xvy7UkFytFBlySOg+d4VOn6y1YWu8ChD4hdjV6J6XouJ4Oilrv6byfrzNuQzQYkFyigfrukvFtXw==" saltValue="p4ztrjlDnXiB32JrIfe5dw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <dataConsolidate/>
   <mergeCells count="115">
     <mergeCell ref="P26:Q26"/>
@@ -40239,16 +40253,16 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7:H14 H20:H34" xr:uid="{58C46DD0-A12A-4113-A125-1ED47F0DD2E4}">
       <formula1>Designation</formula1>
     </dataValidation>
-    <dataValidation type="custom" errorStyle="information" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $225,700 for calandar appointments and $159,871 for academic appointments." sqref="I7:I14 I20:I34" xr:uid="{50F3581B-6538-4C6A-8B28-EC82F3F862AF}">
+    <dataValidation type="custom" errorStyle="information" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $228,000 for calandar appointments and $161,500 for academic appointments." sqref="I20:I34 I7:I14" xr:uid="{50F3581B-6538-4C6A-8B28-EC82F3F862AF}">
       <formula1>IF(AND($O$5="Federal - NIH",OR(NOT(ISBLANK(J7)),NOT(ISBLANK(K7)),NOT(ISBLANK(L7)),J7&lt;&gt;"",K7&lt;&gt;"",L7&lt;&gt;"")),IF(J7&gt;0,I7&lt;=NIHSalaryCap,I7&lt;=(NIHSalaryCap*8.5)/12),TRUE)</formula1>
     </dataValidation>
-    <dataValidation type="custom" errorStyle="information" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $225,700 for calandar appointments and $159,871 for academic appointments." sqref="J7:J14 J20:J34 J53:J72" xr:uid="{09FE9C67-2D1C-4009-81A4-16F4EC97BC4B}">
+    <dataValidation type="custom" errorStyle="information" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $228,000 for calandar appointments and $161,500 for academic appointments." sqref="J53:J72 J7:J14 J20:J34" xr:uid="{09FE9C67-2D1C-4009-81A4-16F4EC97BC4B}">
       <formula1>IF(AND($O$5="Federal - NIH",OR(NOT(ISBLANK(J7)),NOT(ISBLANK(K7)),NOT(ISBLANK(L7)),J7&lt;&gt;"",K7&lt;&gt;"",L7&lt;&gt;"")),IF(J7&gt;0,I7&lt;=NIHSalaryCap,I7&lt;=(NIHSalaryCap*8.5)/12),TRUE)</formula1>
     </dataValidation>
-    <dataValidation type="custom" errorStyle="information" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $225,700 for calandar appointments and $159,871 for academic appointments." sqref="K7:K14 K20:K34 K53:K72" xr:uid="{B8A56B9B-972A-4261-B890-EDF14B88F491}">
+    <dataValidation type="custom" errorStyle="information" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $228,000 for calandar appointments and $161,500 for academic appointments." sqref="K53:K72 K7:K14 K20:K34" xr:uid="{B8A56B9B-972A-4261-B890-EDF14B88F491}">
       <formula1>IF(AND($O$5="Federal - NIH",OR(NOT(ISBLANK(J7)),NOT(ISBLANK(K7)),NOT(ISBLANK(L7)),J7&lt;&gt;"",K7&lt;&gt;"",L7&lt;&gt;"")),IF(J7&gt;0,I7&lt;=NIHSalaryCap,I7&lt;=(NIHSalaryCap*8.5)/12),TRUE)</formula1>
     </dataValidation>
-    <dataValidation type="custom" errorStyle="information" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $225,700 for calandar appointments and $159,871 for academic appointments." sqref="L7:L14 L20:L34 L53:L72" xr:uid="{05BA8183-255B-41B3-9F4E-5F2FE7F28A52}">
+    <dataValidation type="custom" errorStyle="information" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $228,000 for calandar appointments and $161,500 for academic appointments." sqref="L53:L72 L7:L14 L20:L34" xr:uid="{05BA8183-255B-41B3-9F4E-5F2FE7F28A52}">
       <formula1>IF(AND($O$5="Federal - NIH",OR(NOT(ISBLANK(J7)),NOT(ISBLANK(K7)),NOT(ISBLANK(L7)),J7&lt;&gt;"",K7&lt;&gt;"",L7&lt;&gt;"")),IF(J7&gt;0,I7&lt;=NIHSalaryCap,I7&lt;=(NIHSalaryCap*8.5)/12),TRUE)</formula1>
     </dataValidation>
   </dataValidations>
@@ -44578,7 +44592,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="iMv/k2DWT9cS/7DJhrSQlQNZXSpHwRIeMHY0fU1rO1Sv4O1Oj9NiPcTWX9fLP4CGpiruOYNCOxJWuBNOy3OvlA==" saltValue="fWKd9tzbQHT7VCUwSJQZDA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="oER/ByvGraiJDudhtH2Dl7BGozNUgXyijDJ3/c2sERByhFMkanpixOsGD49SHLOGv6xRZ1o+eUN4Ih6KCF7n2Q==" saltValue="uuOP1i1/HJ+MpHP02e2L7A==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <dataConsolidate/>
   <mergeCells count="47">
     <mergeCell ref="I77:M78"/>
@@ -44698,12 +44712,18 @@
       </x14:conditionalFormattings>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="custom" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $225,700 for calandar appointments and $159,871 for academic appointments." xr:uid="{05C536E1-54F3-4A4C-83DA-F9B73EBB6160}">
+          <x14:formula1>
+            <xm:f>IF(AND('Personnel Yr 1'!$O$5="Federal - NIH",OR(NOT(ISBLANK($J20)),NOT(ISBLANK($K20)),NOT(ISBLANK($L20)),$J20&lt;&gt;"",$K20&lt;&gt;"",$L20&lt;&gt;"")),IF($J20&gt;0,$I20&lt;=NIHSalaryCap,$I20&lt;=(NIHSalaryCap*8.5)/12),TRUE)</xm:f>
+          </x14:formula1>
+          <xm:sqref>I20:I34</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="custom" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $228,000 for calandar appointments and $161,500 for academic appointments." xr:uid="{F82CB08D-40FC-4599-B93F-1B746F3A414F}">
           <x14:formula1>
             <xm:f>IF(AND('Personnel Yr 1'!$O$5="Federal - NIH",OR(NOT(ISBLANK($J7)),NOT(ISBLANK($K7)),NOT(ISBLANK($L7)),$J7&lt;&gt;"",$K7&lt;&gt;"",$L7&lt;&gt;"")),IF($J7&gt;0,$I7&lt;=NIHSalaryCap,$I7&lt;=(NIHSalaryCap*8.5)/12),TRUE)</xm:f>
           </x14:formula1>
-          <xm:sqref>I7:L14 I20:L34 J53:L72</xm:sqref>
+          <xm:sqref>I7:L14 I20:L34 J20:L34 J53:L72</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -48983,7 +49003,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="oM6ttyIsOEnDwbQdT0PVDZGJLjeDtWg2js5YnFPgxzMFrXAuCZy42Je2dUSsCHJbDJ82f7b6if0i/mIKpwIxHA==" saltValue="H5JgkWjsF++AIdtbeI0RAw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="fUxUkiPF7IjUfLsC5luL/4xl2k0QY1uwPgYD0fsCEkY98YHklp8SBFVxinDnoYkxqzs3Ufs5D6HiITvMOyv+QA==" saltValue="YE2rz8+MCqYWLDEdj/aBxA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="48">
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="I75:M76"/>
@@ -49104,11 +49124,11 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="custom" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $225,700 for calandar appointments and $159,871 for academic appointments." xr:uid="{A82F715D-55DE-4D42-A3EF-3FEED2DA8D36}">
+        <x14:dataValidation type="custom" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $228,000 for calandar appointments and $161,500 for academic appointments." xr:uid="{A82F715D-55DE-4D42-A3EF-3FEED2DA8D36}">
           <x14:formula1>
             <xm:f>IF(AND('Personnel Yr 1'!$O$5="Federal - NIH",OR(NOT(ISBLANK($J7)),NOT(ISBLANK($K7)),NOT(ISBLANK($L7)),$J7&lt;&gt;"",$K7&lt;&gt;"",$L7&lt;&gt;"")),IF($J7&gt;0,$I7&lt;=NIHSalaryCap,$I7&lt;=(NIHSalaryCap*8.5)/12),TRUE)</xm:f>
           </x14:formula1>
-          <xm:sqref>I7:L14 I20:L34 J53:L72</xm:sqref>
+          <xm:sqref>J53:L72 I7:L14 I20:L34</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -53381,7 +53401,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="YIt/qtEwh2OD8GQ6y34qPJflY0WFImCWRmPsMfd+h7G+F8wg0PgXNC4GWXiqNJxbk86p6IMU5Ps80l15FF0YEA==" saltValue="xIWolZwdBF4dlcPSUQPk4A==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="GBVoGZy1R/1F2nIC+BHP4JV88sX1FcP428oLSHoU5G3AVLAne6LY+jfJHb2RqMo/a+0zPXdI/CvBUglEXqiw9g==" saltValue="e7kxP7QT57OmciqzbifTEw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="48">
     <mergeCell ref="C43:F43"/>
     <mergeCell ref="C47:I47"/>
@@ -53505,11 +53525,11 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="custom" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $225,700 for calandar appointments and $159,871 for academic appointments." xr:uid="{EF98792D-7C1E-45E1-BE2E-3DBE7916E6FB}">
+        <x14:dataValidation type="custom" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $228,000 for calandar appointments and $161,500 for academic appointments." xr:uid="{EF98792D-7C1E-45E1-BE2E-3DBE7916E6FB}">
           <x14:formula1>
             <xm:f>IF(AND('Personnel Yr 1'!$O$5="Federal - NIH",OR(NOT(ISBLANK($J7)),NOT(ISBLANK($K7)),NOT(ISBLANK($L7)),$J7&lt;&gt;"",$K7&lt;&gt;"",$L7&lt;&gt;"")),IF($J7&gt;0,$I7&lt;=NIHSalaryCap,$I7&lt;=(NIHSalaryCap*8.5)/12),TRUE)</xm:f>
           </x14:formula1>
-          <xm:sqref>I7:L14 I20:L34 J53:L72</xm:sqref>
+          <xm:sqref>J53:L72 I7:L14 I20:L34</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -58627,7 +58647,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="/GynPkepHmYhdjuCLvCu85XP/T7rpUmIDSjFwpo7xDrIo/sKCrVNn0LGFcMR4Ch3omJnkf2LeuTfx+HewX31JA==" saltValue="JyaVwBnAWisIR5R4ZCh/Mw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="zG/E1XjpgQ6Ipt/NuEhU7BXyoztj503Dgg+Pg9WXXQ0fpYSa9/l4tZjRSp8re4c9aMziy651429DL1OT3aFXjA==" saltValue="JzY3BKJvEzliqfZhbDBjnw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="47">
     <mergeCell ref="C43:F43"/>
     <mergeCell ref="C47:I47"/>
@@ -58747,11 +58767,11 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="custom" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $225,700 for calandar appointments and $159,871 for academic appointments." xr:uid="{14F9BA64-990C-4EE1-95E1-54F956BE092C}">
+        <x14:dataValidation type="custom" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Salary Cap Error" error="Base salary should remain under $228,000 for calandar appointments and $161,500 for academic appointments." xr:uid="{14F9BA64-990C-4EE1-95E1-54F956BE092C}">
           <x14:formula1>
             <xm:f>IF(AND('Personnel Yr 1'!$O$5="Federal - NIH",OR(NOT(ISBLANK($J7)),NOT(ISBLANK($K7)),NOT(ISBLANK($L7)),$J7&lt;&gt;"",$K7&lt;&gt;"",$L7&lt;&gt;"")),IF($J7&gt;0,$I7&lt;=NIHSalaryCap,$I7&lt;=(NIHSalaryCap*8.5)/12),TRUE)</xm:f>
           </x14:formula1>
-          <xm:sqref>I7:L14 I20:L34 J53:L72</xm:sqref>
+          <xm:sqref>J53:L72 I7:L14 I20:L34</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>